<commit_message>
fixed: correct_answer mapping added: question id asauto incrementing number
</commit_message>
<xml_diff>
--- a/entrytestguru/assets/templates/bulk_upload_template.xlsx
+++ b/entrytestguru/assets/templates/bulk_upload_template.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Non_Office\Dev_Space\vibe_skool\etg-code\entrytestguru\assets\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5586306-3E4D-4848-BC6B-9083A79FDBFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB8A9D89-AA40-4FCD-9A03-7B6D0136C9D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{3DE5D032-E4C7-45AF-B710-A9735A21A42C}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="20640" windowHeight="11040" xr2:uid="{3DE5D032-E4C7-45AF-B710-A9735A21A42C}"/>
   </bookViews>
   <sheets>
     <sheet name="bulk_upload_template" sheetId="1" r:id="rId1"/>
     <sheet name="lookups" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">bulk_upload_template!$A$1:$T$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">bulk_upload_template!$B$1:$U$20</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="492">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="500">
   <si>
     <t>questionText</t>
   </si>
@@ -1537,6 +1537,30 @@
   </si>
   <si>
     <t>To solve the linear equation 3x-5=13, you must isolate the variable x. First, add 5 to both sides of the equation: 3x-5+5=13+5, which simplifies to 3x=18.Next, divide both sides by 3 to find the value of x: 3x/3=18/3, which gives x=6.</t>
+  </si>
+  <si>
+    <t>questionId</t>
+  </si>
+  <si>
+    <t>if f(x)=81, then what is the degree of the function f(x)</t>
+  </si>
+  <si>
+    <t>liner</t>
+  </si>
+  <si>
+    <t>quadratic</t>
+  </si>
+  <si>
+    <t>cubic</t>
+  </si>
+  <si>
+    <t>exponential</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>lorem ipsum dah dah dah</t>
   </si>
 </sst>
 </file>
@@ -1902,7 +1926,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -2032,6 +2056,19 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -2077,7 +2114,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2099,11 +2136,17 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -2480,1086 +2523,1218 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B50BA1B2-A2A0-43CA-A45C-69B9256BF234}">
-  <dimension ref="A1:U20"/>
+  <dimension ref="A1:V21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="38.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.140625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="13.85546875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="12.7109375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="13.140625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="11.140625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="12" style="1" customWidth="1"/>
-    <col min="13" max="13" width="9.42578125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="67.28515625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="14.28515625" style="1" customWidth="1"/>
-    <col min="16" max="16" width="10.28515625" style="1" customWidth="1"/>
-    <col min="17" max="17" width="15.85546875" style="1" customWidth="1"/>
-    <col min="18" max="18" width="16.7109375" style="1" customWidth="1"/>
-    <col min="19" max="19" width="18.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="19.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="9.140625" style="1"/>
+    <col min="2" max="2" width="38.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="16" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.140625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="13.85546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.140625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="11.140625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="12" style="1" customWidth="1"/>
+    <col min="14" max="14" width="9.42578125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="67.28515625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="14.28515625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="10.28515625" style="1" customWidth="1"/>
+    <col min="18" max="18" width="15.85546875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="16.7109375" style="1" customWidth="1"/>
+    <col min="20" max="20" width="18.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="19.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="B1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="12"/>
-    </row>
-    <row r="2" spans="1:21" ht="60" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="V1" s="12"/>
+    </row>
+    <row r="2" spans="1:22" ht="60" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>457</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>424</v>
       </c>
-      <c r="H2" s="2">
+      <c r="I2" s="2">
         <v>6</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>425</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>426</v>
       </c>
-      <c r="K2" s="2"/>
       <c r="L2" s="2"/>
-      <c r="M2" s="2" t="str">
+      <c r="M2" s="2"/>
+      <c r="N2" s="2" t="str">
         <f ca="1">CHAR(RANDBETWEEN(65,68))</f>
         <v>D</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="O2" s="2" t="s">
         <v>491</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="P2" s="2" t="s">
         <v>427</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="Q2" s="2" t="s">
         <v>428</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="R2" s="2">
         <v>60</v>
       </c>
-      <c r="R2" s="2">
+      <c r="S2" s="2">
         <v>0.9</v>
       </c>
-      <c r="S2" s="2"/>
       <c r="T2" s="2"/>
-    </row>
-    <row r="3" spans="1:21" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="U2" s="2"/>
+    </row>
+    <row r="3" spans="1:22" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <f>A2+1</f>
+        <v>2</v>
+      </c>
+      <c r="B3" s="15" t="s">
         <v>429</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>430</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>431</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="J3" s="2" t="s">
         <v>432</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="K3" s="2" t="s">
         <v>433</v>
       </c>
-      <c r="K3" s="2"/>
       <c r="L3" s="2"/>
-      <c r="M3" s="2" t="str">
-        <f t="shared" ref="M3:M20" ca="1" si="0">CHAR(RANDBETWEEN(65,68))</f>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2" t="str">
+        <f t="shared" ref="N3:N20" ca="1" si="0">CHAR(RANDBETWEEN(65,68))</f>
+        <v>B</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="R3" s="2">
+        <v>120</v>
+      </c>
+      <c r="S3" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="T3" s="2"/>
+      <c r="U3" s="2"/>
+    </row>
+    <row r="4" spans="1:22" ht="60" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <f t="shared" ref="A4:A20" si="1">A3+1</f>
+        <v>3</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>436</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2" t="str">
+        <f t="shared" ca="1" si="0"/>
         <v>C</v>
       </c>
-      <c r="N3" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="O3" s="2" t="s">
+      <c r="O4" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="P4" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="Q4" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="R4" s="2">
+        <v>150</v>
+      </c>
+      <c r="S4" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="T4" s="2"/>
+      <c r="U4" s="2"/>
+    </row>
+    <row r="5" spans="1:22" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>443</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>B</v>
+      </c>
+      <c r="O5" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="P5" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="Q5" s="2" t="s">
         <v>428</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="R5" s="2">
+        <v>90</v>
+      </c>
+      <c r="S5" s="2">
+        <v>0.9</v>
+      </c>
+      <c r="T5" s="2"/>
+      <c r="U5" s="2"/>
+    </row>
+    <row r="6" spans="1:22" ht="60" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>449</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" s="2">
+        <v>17</v>
+      </c>
+      <c r="I6" s="2">
+        <v>19</v>
+      </c>
+      <c r="J6" s="2">
+        <v>15</v>
+      </c>
+      <c r="K6" s="2">
+        <v>21</v>
+      </c>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>C</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="Q6" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="R6" s="2">
         <v>120</v>
       </c>
-      <c r="R3" s="2">
+      <c r="S6" s="2">
         <v>0.8</v>
       </c>
-      <c r="S3" s="2"/>
-      <c r="T3" s="2"/>
-    </row>
-    <row r="4" spans="1:21" ht="60" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>436</v>
-      </c>
-      <c r="B4" s="2" t="s">
+      <c r="T6" s="2"/>
+      <c r="U6" s="2"/>
+    </row>
+    <row r="7" spans="1:22" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>451</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>437</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>439</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>440</v>
-      </c>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2" t="str">
+      <c r="E7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>D</v>
       </c>
-      <c r="N4" s="2" t="s">
-        <v>441</v>
-      </c>
-      <c r="O4" s="2" t="s">
-        <v>435</v>
-      </c>
-      <c r="P4" s="2" t="s">
-        <v>442</v>
-      </c>
-      <c r="Q4" s="2">
-        <v>150</v>
-      </c>
-      <c r="R4" s="2">
-        <v>0.8</v>
-      </c>
-      <c r="S4" s="2"/>
-      <c r="T4" s="2"/>
-    </row>
-    <row r="5" spans="1:21" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>443</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>444</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>445</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>446</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>447</v>
-      </c>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>B</v>
-      </c>
-      <c r="N5" s="2" t="s">
-        <v>448</v>
-      </c>
-      <c r="O5" s="2" t="s">
-        <v>427</v>
-      </c>
-      <c r="P5" s="2" t="s">
-        <v>428</v>
-      </c>
-      <c r="Q5" s="2">
-        <v>90</v>
-      </c>
-      <c r="R5" s="2">
-        <v>0.9</v>
-      </c>
-      <c r="S5" s="2"/>
-      <c r="T5" s="2"/>
-    </row>
-    <row r="6" spans="1:21" ht="60" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>449</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" s="2">
-        <v>17</v>
-      </c>
-      <c r="H6" s="2">
-        <v>19</v>
-      </c>
-      <c r="I6" s="2">
-        <v>15</v>
-      </c>
-      <c r="J6" s="2">
-        <v>21</v>
-      </c>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>D</v>
-      </c>
-      <c r="N6" s="2" t="s">
-        <v>450</v>
-      </c>
-      <c r="O6" s="2" t="s">
-        <v>435</v>
-      </c>
-      <c r="P6" s="2" t="s">
-        <v>442</v>
-      </c>
-      <c r="Q6" s="2">
-        <v>120</v>
-      </c>
-      <c r="R6" s="2">
-        <v>0.8</v>
-      </c>
-      <c r="S6" s="2"/>
-      <c r="T6" s="2"/>
-    </row>
-    <row r="7" spans="1:21" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
-        <v>451</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>452</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>453</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>454</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>A</v>
-      </c>
-      <c r="N7" s="2" t="s">
+      <c r="O7" s="2" t="s">
         <v>458</v>
       </c>
-      <c r="O7" s="2" t="s">
+      <c r="P7" s="2" t="s">
         <v>456</v>
       </c>
-      <c r="P7" s="2"/>
       <c r="Q7" s="2"/>
       <c r="R7" s="2"/>
       <c r="S7" s="2"/>
       <c r="T7" s="2"/>
-    </row>
-    <row r="8" spans="1:21" ht="60" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="U7" s="2"/>
+    </row>
+    <row r="8" spans="1:22" ht="60" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>469</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>21</v>
       </c>
       <c r="G8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" s="1" t="s">
         <v>459</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="I8" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="J8" s="1" t="s">
         <v>465</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="K8" s="1" t="s">
         <v>466</v>
       </c>
-      <c r="M8" s="2" t="str">
+      <c r="N8" s="2" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>D</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="P8" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="Q8" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="R8" s="1">
+        <v>149</v>
+      </c>
+      <c r="S8" s="1">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="N9" s="2" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>C</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="P9" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="Q9" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="R9" s="1">
+        <v>97</v>
+      </c>
+      <c r="S9" s="1">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H10" s="1">
+        <v>25</v>
+      </c>
+      <c r="I10" s="1">
+        <v>20</v>
+      </c>
+      <c r="J10" s="1">
+        <v>30</v>
+      </c>
+      <c r="K10" s="1">
+        <v>15</v>
+      </c>
+      <c r="N10" s="2" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>B</v>
       </c>
-      <c r="N8" s="1" t="s">
-        <v>470</v>
-      </c>
-      <c r="O8" s="1" t="s">
+      <c r="O10" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="P10" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="Q10" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="R10" s="1">
+        <v>75</v>
+      </c>
+      <c r="S10" s="1">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="N11" s="2" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>A</v>
+      </c>
+      <c r="O11" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="P11" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="P8" s="1" t="s">
+      <c r="Q11" s="1" t="s">
         <v>467</v>
       </c>
-      <c r="Q8" s="1">
-        <v>149</v>
-      </c>
-      <c r="R8" s="1">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:21" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>471</v>
-      </c>
-      <c r="B9" s="1" t="s">
+      <c r="R11" s="1">
+        <v>94</v>
+      </c>
+      <c r="S11" s="1">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" ht="60" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <f t="shared" si="1"/>
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D12" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="1" t="s">
-        <v>466</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>465</v>
-      </c>
-      <c r="I9" s="1" t="s">
-        <v>459</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>464</v>
-      </c>
-      <c r="M9" s="2" t="str">
+      <c r="H12" s="1">
+        <v>25</v>
+      </c>
+      <c r="I12" s="1">
+        <v>30</v>
+      </c>
+      <c r="J12" s="1">
+        <v>20</v>
+      </c>
+      <c r="K12" s="1">
+        <v>15</v>
+      </c>
+      <c r="N12" s="2" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>B</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="P12" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="Q12" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="R12" s="1">
+        <v>162</v>
+      </c>
+      <c r="S12" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" ht="60" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <f t="shared" si="1"/>
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H13" s="1">
+        <v>20</v>
+      </c>
+      <c r="I13" s="1">
+        <v>25</v>
+      </c>
+      <c r="J13" s="1">
+        <v>15</v>
+      </c>
+      <c r="K13" s="1">
+        <v>30</v>
+      </c>
+      <c r="N13" s="2" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>D</v>
       </c>
-      <c r="N9" s="1" t="s">
-        <v>472</v>
-      </c>
-      <c r="O9" s="1" t="s">
+      <c r="O13" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="P13" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="Q13" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="R13" s="1">
+        <v>116</v>
+      </c>
+      <c r="S13" s="1">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <f t="shared" si="1"/>
+        <v>13</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H14" s="1">
+        <v>30</v>
+      </c>
+      <c r="I14" s="1">
+        <v>15</v>
+      </c>
+      <c r="J14" s="1">
+        <v>20</v>
+      </c>
+      <c r="K14" s="1">
+        <v>25</v>
+      </c>
+      <c r="N14" s="2" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>C</v>
+      </c>
+      <c r="O14" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="P14" s="1" t="s">
         <v>427</v>
       </c>
-      <c r="P9" s="1" t="s">
+      <c r="Q14" s="1" t="s">
         <v>467</v>
       </c>
-      <c r="Q9" s="1">
-        <v>97</v>
-      </c>
-      <c r="R9" s="1">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>473</v>
-      </c>
-      <c r="B10" s="1" t="s">
+      <c r="R14" s="1">
+        <v>166</v>
+      </c>
+      <c r="S14" s="1">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
+        <f t="shared" si="1"/>
+        <v>14</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>481</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="D15" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="E15" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F15" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G10" s="1">
+      <c r="H15" s="1">
+        <v>15</v>
+      </c>
+      <c r="I15" s="1">
+        <v>20</v>
+      </c>
+      <c r="J15" s="1">
+        <v>30</v>
+      </c>
+      <c r="K15" s="1">
         <v>25</v>
       </c>
-      <c r="H10" s="1">
-        <v>20</v>
-      </c>
-      <c r="I10" s="1">
-        <v>30</v>
-      </c>
-      <c r="J10" s="1">
-        <v>15</v>
-      </c>
-      <c r="M10" s="2" t="str">
+      <c r="N15" s="2" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>D</v>
       </c>
-      <c r="N10" s="1" t="s">
+      <c r="O15" s="1" t="s">
         <v>474</v>
       </c>
-      <c r="O10" s="1" t="s">
-        <v>427</v>
-      </c>
-      <c r="P10" s="1" t="s">
+      <c r="P15" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="Q15" s="1" t="s">
         <v>467</v>
       </c>
-      <c r="Q10" s="1">
-        <v>75</v>
-      </c>
-      <c r="R10" s="1">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>475</v>
-      </c>
-      <c r="B11" s="1" t="s">
+      <c r="R15" s="1">
+        <v>124</v>
+      </c>
+      <c r="S15" s="1">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22" ht="45" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="D16" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="E16" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G11" s="1" t="s">
-        <v>465</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>459</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>466</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>464</v>
-      </c>
-      <c r="M11" s="2" t="str">
+      <c r="H16" s="1">
+        <f>-2/3</f>
+        <v>-0.66666666666666663</v>
+      </c>
+      <c r="I16" s="1">
+        <f>-1/4</f>
+        <v>-0.25</v>
+      </c>
+      <c r="J16" s="13">
+        <v>45750</v>
+      </c>
+      <c r="K16" s="13">
+        <v>45689</v>
+      </c>
+      <c r="N16" s="2" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>C</v>
+      </c>
+      <c r="O16" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="P16" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="Q16" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="R16" s="1">
+        <v>86</v>
+      </c>
+      <c r="S16" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <f t="shared" si="1"/>
+        <v>16</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H17" s="1">
+        <v>30</v>
+      </c>
+      <c r="I17" s="1">
+        <v>25</v>
+      </c>
+      <c r="J17" s="1">
+        <v>15</v>
+      </c>
+      <c r="K17" s="1">
+        <v>20</v>
+      </c>
+      <c r="N17" s="2" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>A</v>
       </c>
-      <c r="N11" s="1" t="s">
-        <v>472</v>
-      </c>
-      <c r="O11" s="1" t="s">
+      <c r="O17" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="P17" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="Q17" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="R17" s="1">
+        <v>104</v>
+      </c>
+      <c r="S17" s="1">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
+        <f t="shared" si="1"/>
+        <v>17</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H18" s="1">
+        <v>25</v>
+      </c>
+      <c r="I18" s="1">
+        <v>30</v>
+      </c>
+      <c r="J18" s="1">
+        <v>15</v>
+      </c>
+      <c r="K18" s="1">
+        <v>20</v>
+      </c>
+      <c r="N18" s="2" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>D</v>
+      </c>
+      <c r="O18" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="P18" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="P11" s="1" t="s">
-        <v>467</v>
-      </c>
-      <c r="Q11" s="1">
-        <v>94</v>
-      </c>
-      <c r="R11" s="1">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21" ht="60" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>476</v>
-      </c>
-      <c r="B12" s="1" t="s">
+      <c r="Q18" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="R18" s="1">
+        <v>128</v>
+      </c>
+      <c r="S18" s="1">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+      <c r="A19" s="2">
+        <f t="shared" si="1"/>
+        <v>18</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="D19" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="E19" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G12" s="1">
+      <c r="F19" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H19" s="1">
+        <v>20</v>
+      </c>
+      <c r="I19" s="1">
+        <v>15</v>
+      </c>
+      <c r="J19" s="1">
         <v>25</v>
       </c>
-      <c r="H12" s="1">
+      <c r="K19" s="1">
         <v>30</v>
       </c>
-      <c r="I12" s="1">
-        <v>20</v>
-      </c>
-      <c r="J12" s="1">
-        <v>15</v>
-      </c>
-      <c r="M12" s="2" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>A</v>
-      </c>
-      <c r="N12" s="1" t="s">
-        <v>477</v>
-      </c>
-      <c r="O12" s="1" t="s">
-        <v>456</v>
-      </c>
-      <c r="P12" s="1" t="s">
-        <v>467</v>
-      </c>
-      <c r="Q12" s="1">
-        <v>162</v>
-      </c>
-      <c r="R12" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:21" ht="60" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>478</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G13" s="1">
-        <v>20</v>
-      </c>
-      <c r="H13" s="1">
-        <v>25</v>
-      </c>
-      <c r="I13" s="1">
-        <v>15</v>
-      </c>
-      <c r="J13" s="1">
-        <v>30</v>
-      </c>
-      <c r="M13" s="2" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>B</v>
-      </c>
-      <c r="N13" s="1" t="s">
-        <v>479</v>
-      </c>
-      <c r="O13" s="1" t="s">
-        <v>456</v>
-      </c>
-      <c r="P13" s="1" t="s">
-        <v>467</v>
-      </c>
-      <c r="Q13" s="1">
-        <v>116</v>
-      </c>
-      <c r="R13" s="1">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:21" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>480</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G14" s="1">
-        <v>30</v>
-      </c>
-      <c r="H14" s="1">
-        <v>15</v>
-      </c>
-      <c r="I14" s="1">
-        <v>20</v>
-      </c>
-      <c r="J14" s="1">
-        <v>25</v>
-      </c>
-      <c r="M14" s="2" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>A</v>
-      </c>
-      <c r="N14" s="1" t="s">
-        <v>474</v>
-      </c>
-      <c r="O14" s="1" t="s">
-        <v>427</v>
-      </c>
-      <c r="P14" s="1" t="s">
-        <v>467</v>
-      </c>
-      <c r="Q14" s="1">
-        <v>166</v>
-      </c>
-      <c r="R14" s="1">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:21" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>481</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G15" s="1">
-        <v>15</v>
-      </c>
-      <c r="H15" s="1">
-        <v>20</v>
-      </c>
-      <c r="I15" s="1">
-        <v>30</v>
-      </c>
-      <c r="J15" s="1">
-        <v>25</v>
-      </c>
-      <c r="M15" s="2" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>B</v>
-      </c>
-      <c r="N15" s="1" t="s">
-        <v>474</v>
-      </c>
-      <c r="O15" s="1" t="s">
-        <v>456</v>
-      </c>
-      <c r="P15" s="1" t="s">
-        <v>467</v>
-      </c>
-      <c r="Q15" s="1">
-        <v>124</v>
-      </c>
-      <c r="R15" s="1">
-        <v>0.7</v>
-      </c>
-    </row>
-    <row r="16" spans="1:21" ht="45" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>482</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G16" s="1">
-        <f>-2/3</f>
-        <v>-0.66666666666666663</v>
-      </c>
-      <c r="H16" s="1">
-        <f>-1/4</f>
-        <v>-0.25</v>
-      </c>
-      <c r="I16" s="14">
-        <v>45750</v>
-      </c>
-      <c r="J16" s="14">
-        <v>45689</v>
-      </c>
-      <c r="M16" s="2" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>A</v>
-      </c>
-      <c r="N16" s="1" t="s">
-        <v>483</v>
-      </c>
-      <c r="O16" s="1" t="s">
-        <v>435</v>
-      </c>
-      <c r="P16" s="1" t="s">
-        <v>467</v>
-      </c>
-      <c r="Q16" s="1">
-        <v>86</v>
-      </c>
-      <c r="R16" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:18" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>484</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G17" s="1">
-        <v>30</v>
-      </c>
-      <c r="H17" s="1">
-        <v>25</v>
-      </c>
-      <c r="I17" s="1">
-        <v>15</v>
-      </c>
-      <c r="J17" s="1">
-        <v>20</v>
-      </c>
-      <c r="M17" s="2" t="str">
+      <c r="N19" s="2" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>C</v>
       </c>
-      <c r="N17" s="1" t="s">
-        <v>474</v>
-      </c>
-      <c r="O17" s="1" t="s">
+      <c r="O19" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="P19" s="1" t="s">
         <v>427</v>
       </c>
-      <c r="P17" s="1" t="s">
-        <v>467</v>
-      </c>
-      <c r="Q17" s="1">
-        <v>104</v>
-      </c>
-      <c r="R17" s="1">
-        <v>0.7</v>
-      </c>
-    </row>
-    <row r="18" spans="1:18" ht="45" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>485</v>
-      </c>
-      <c r="B18" s="1" t="s">
+      <c r="Q19" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="R19" s="1">
+        <v>164</v>
+      </c>
+      <c r="S19" s="1">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+      <c r="A20" s="2">
+        <f t="shared" si="1"/>
+        <v>19</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="D20" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="E20" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="F20" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="G20" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G18" s="1">
+      <c r="H20" s="1">
+        <v>15</v>
+      </c>
+      <c r="I20" s="1">
+        <v>30</v>
+      </c>
+      <c r="J20" s="1">
+        <v>20</v>
+      </c>
+      <c r="K20" s="1">
         <v>25</v>
       </c>
-      <c r="H18" s="1">
-        <v>30</v>
-      </c>
-      <c r="I18" s="1">
-        <v>15</v>
-      </c>
-      <c r="J18" s="1">
-        <v>20</v>
-      </c>
-      <c r="M18" s="2" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>A</v>
-      </c>
-      <c r="N18" s="1" t="s">
-        <v>486</v>
-      </c>
-      <c r="O18" s="1" t="s">
-        <v>435</v>
-      </c>
-      <c r="P18" s="1" t="s">
-        <v>468</v>
-      </c>
-      <c r="Q18" s="1">
-        <v>128</v>
-      </c>
-      <c r="R18" s="1">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="19" spans="1:18" ht="60" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>487</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="G19" s="1">
-        <v>20</v>
-      </c>
-      <c r="H19" s="1">
-        <v>15</v>
-      </c>
-      <c r="I19" s="1">
-        <v>25</v>
-      </c>
-      <c r="J19" s="1">
-        <v>30</v>
-      </c>
-      <c r="M19" s="2" t="str">
+      <c r="N20" s="2" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>D</v>
       </c>
-      <c r="N19" s="1" t="s">
-        <v>488</v>
-      </c>
-      <c r="O19" s="1" t="s">
+      <c r="O20" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="P20" s="1" t="s">
         <v>427</v>
       </c>
-      <c r="P19" s="1" t="s">
+      <c r="Q20" s="1" t="s">
         <v>468</v>
       </c>
-      <c r="Q19" s="1">
-        <v>164</v>
-      </c>
-      <c r="R19" s="1">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="20" spans="1:18" ht="45" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>489</v>
-      </c>
-      <c r="B20" s="1" t="s">
+      <c r="R20" s="1">
+        <v>87</v>
+      </c>
+      <c r="S20" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>20</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="D21" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="E21" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="F21" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="G21" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="G20" s="1">
-        <v>15</v>
-      </c>
-      <c r="H20" s="1">
-        <v>30</v>
-      </c>
-      <c r="I20" s="1">
-        <v>20</v>
-      </c>
-      <c r="J20" s="1">
-        <v>25</v>
-      </c>
-      <c r="M20" s="2" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>A</v>
-      </c>
-      <c r="N20" s="1" t="s">
-        <v>490</v>
-      </c>
-      <c r="O20" s="1" t="s">
+      <c r="H21" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>495</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>497</v>
+      </c>
+      <c r="N21" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="O21" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="P21" s="1" t="s">
         <v>427</v>
       </c>
-      <c r="P20" s="1" t="s">
+      <c r="Q21" s="1" t="s">
         <v>468</v>
       </c>
-      <c r="Q20" s="1">
-        <v>87</v>
-      </c>
-      <c r="R20" s="1">
-        <v>1</v>
+      <c r="R21" s="1">
+        <v>5</v>
+      </c>
+      <c r="S21" s="1">
+        <v>0.05</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T20" xr:uid="{B50BA1B2-A2A0-43CA-A45C-69B9256BF234}"/>
+  <autoFilter ref="B1:U20" xr:uid="{B50BA1B2-A2A0-43CA-A45C-69B9256BF234}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -3568,31 +3743,31 @@
           <x14:formula1>
             <xm:f>lookups!$C$2:$C$3</xm:f>
           </x14:formula1>
-          <xm:sqref>B2:B7 B14:B20</xm:sqref>
+          <xm:sqref>C2:C7 C14:C21</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{C3745A5F-A079-40F8-89D6-D2CBD53DE1B7}">
           <x14:formula1>
             <xm:f>lookups!$A$2:$A$7</xm:f>
           </x14:formula1>
-          <xm:sqref>C2:C7 C14:C20</xm:sqref>
+          <xm:sqref>D2:D7 D14:D21</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EDA5A3DB-F736-4A7F-BD94-30556C13E5D0}">
           <x14:formula1>
             <xm:f>lookups!$G$2:$G$117</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E7 E14:E20</xm:sqref>
+          <xm:sqref>F2:F7 F14:F21</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{1CE0BA8D-60F5-4392-8D81-75B3DCD3988C}">
           <x14:formula1>
             <xm:f>lookups!$E$2:$E$6</xm:f>
           </x14:formula1>
-          <xm:sqref>D2:D7 D14:D20</xm:sqref>
+          <xm:sqref>E2:E7 E14:E21</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D9A4D77F-881D-4C85-B4B6-FD00BD6C9DF3}">
           <x14:formula1>
             <xm:f>lookups!$I$2:$I$300</xm:f>
           </x14:formula1>
-          <xm:sqref>F2:F7 F14:F20</xm:sqref>
+          <xm:sqref>G2:G7 G14:G21</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>